<commit_message>
Update Issues Log: fix rows 2, 5, 8, 9, 10, add row 16
</commit_message>
<xml_diff>
--- a/excel/issues_log.xlsx
+++ b/excel/issues_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DEIVI\Desktop\DA Projects\delivery-performance-analysis\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F01B1BC2-DB64-4C9C-AA5D-C6EB74126C52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E658DEF0-A46F-4036-9784-3C3ED00CC949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-27" yWindow="0" windowWidth="20581" windowHeight="19657" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="103">
   <si>
     <t>lines</t>
   </si>
@@ -52,9 +52,6 @@
     <t>fixed in</t>
   </si>
   <si>
-    <t>TBD</t>
-  </si>
-  <si>
     <t>Delivery Status, Late_delivery_risk, Days for shipping (real), Days for shipment (scheduled)</t>
   </si>
   <si>
@@ -97,9 +94,6 @@
     <t>Query 5a</t>
   </si>
   <si>
-    <t>Planned: clean step</t>
-  </si>
-  <si>
     <t>Canceled lines include suspected-fraud orders</t>
   </si>
   <si>
@@ -271,9 +265,6 @@
     <t>Jan 2015 to Oct 2017: about 5,200 lines and 1,750 orders a month. Oct 2017 to Jan 2018: 8,557 lines, 8,403 orders</t>
   </si>
   <si>
-    <t>Order volume did not drop (about 1,750 to about 2,100 a month); only the line count did. From Nov 2017 each order is a single line</t>
-  </si>
-  <si>
     <t>N/A: No KPI uses them.</t>
   </si>
   <si>
@@ -298,9 +289,6 @@
     <t>05_model.sql</t>
   </si>
   <si>
-    <t>05_model.sql.</t>
-  </si>
-  <si>
     <t>One category listed under two departments</t>
   </si>
   <si>
@@ -317,6 +305,36 @@
   </si>
   <si>
     <t>Step 11 test</t>
+  </si>
+  <si>
+    <t>Order Country, Order Region</t>
+  </si>
+  <si>
+    <t>Order State, Order City</t>
+  </si>
+  <si>
+    <t>Every later KPI must reconcile to this baseline</t>
+  </si>
+  <si>
+    <t>Order volume did not drop (about 1,750 to 2,100 a month)</t>
+  </si>
+  <si>
+    <t>Monthly order volume steps up about 20% from Oct 2017</t>
+  </si>
+  <si>
+    <t>8,043 orders, Oct 2017 to Jan 2018 (about 2,000 a month vs about 1,650 before)</t>
+  </si>
+  <si>
+    <t>Report the late rate; do not report volume trends across Oct 2017</t>
+  </si>
+  <si>
+    <t>The late rate stayed at 56 to 59% through the change, so the rate is comparable across the whole period; the volume change is not explained by the data</t>
+  </si>
+  <si>
+    <t>KPI 2</t>
+  </si>
+  <si>
+    <t>N/A: no data change</t>
   </si>
 </sst>
 </file>
@@ -674,36 +692,36 @@
         <v>6</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="85.6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="71.349999999999994" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>83</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="57.1" x14ac:dyDescent="0.25">
@@ -711,25 +729,25 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="H3" s="2" t="s">
-        <v>8</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="42.8" x14ac:dyDescent="0.25">
@@ -737,25 +755,25 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="H4" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="71.349999999999994" x14ac:dyDescent="0.25">
@@ -763,25 +781,25 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="H5" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="42.8" x14ac:dyDescent="0.25">
@@ -789,25 +807,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D6" s="2">
         <v>0</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>34</v>
-      </c>
       <c r="H6" s="2" t="s">
-        <v>23</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="42.8" x14ac:dyDescent="0.25">
@@ -815,25 +833,25 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="H7" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="57.1" x14ac:dyDescent="0.25">
@@ -841,25 +859,25 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="42.8" x14ac:dyDescent="0.25">
@@ -867,21 +885,23 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>46</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="57.1" x14ac:dyDescent="0.25">
@@ -889,21 +909,23 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C10" s="2"/>
+        <v>46</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>93</v>
+      </c>
       <c r="D10" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="28.55" x14ac:dyDescent="0.25">
@@ -911,21 +933,23 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E11" t="s">
         <v>52</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E11" t="s">
-        <v>54</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="42.8" x14ac:dyDescent="0.25">
@@ -933,25 +957,25 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="57.1" x14ac:dyDescent="0.25">
@@ -959,25 +983,25 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D13" s="3">
         <v>180519</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="42.8" x14ac:dyDescent="0.25">
@@ -985,25 +1009,25 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D14" s="3">
         <v>180519</v>
       </c>
       <c r="E14" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="H14" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.25">
@@ -1011,25 +1035,25 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D15" s="3">
         <v>180519</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
@@ -1037,36 +1061,52 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="H16" s="2" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
+        <v>86</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="99.85" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
@@ -1314,13 +1354,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update issues log: rows 8, 9 , 10
</commit_message>
<xml_diff>
--- a/excel/issues_log.xlsx
+++ b/excel/issues_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DEIVI\Desktop\DA Projects\delivery-performance-analysis\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E658DEF0-A46F-4036-9784-3C3ED00CC949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3E4C9E6-BBBF-4F4C-8B65-EB98902F88B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-27" yWindow="0" windowWidth="20581" windowHeight="19657" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="106">
   <si>
     <t>lines</t>
   </si>
@@ -175,9 +175,6 @@
     <t>Query 8c</t>
   </si>
   <si>
-    <t>24,840 Estados Unidos lines (count them with a filter if you want a number)</t>
-  </si>
-  <si>
     <t>Baseline size: one row per item, not per order</t>
   </si>
   <si>
@@ -265,9 +262,6 @@
     <t>Jan 2015 to Oct 2017: about 5,200 lines and 1,750 orders a month. Oct 2017 to Jan 2018: 8,557 lines, 8,403 orders</t>
   </si>
   <si>
-    <t>N/A: No KPI uses them.</t>
-  </si>
-  <si>
     <t>Count KPIs per order</t>
   </si>
   <si>
@@ -335,6 +329,21 @@
   </si>
   <si>
     <t>N/A: no data change</t>
+  </si>
+  <si>
+    <t>No KPI uses them; translating would add effort for no result</t>
+  </si>
+  <si>
+    <t>N/A: no KPI uses them</t>
+  </si>
+  <si>
+    <t>24,840 Estados Unidos lines</t>
+  </si>
+  <si>
+    <t>Country alone would join one country to 4 regions and duplicate rows</t>
+  </si>
+  <si>
+    <t>Order Id, Order Item Id</t>
   </si>
 </sst>
 </file>
@@ -703,25 +712,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="57.1" x14ac:dyDescent="0.25">
@@ -747,7 +756,7 @@
         <v>15</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="42.8" x14ac:dyDescent="0.25">
@@ -773,7 +782,7 @@
         <v>21</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="71.349999999999994" x14ac:dyDescent="0.25">
@@ -799,7 +808,7 @@
         <v>27</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="42.8" x14ac:dyDescent="0.25">
@@ -825,7 +834,7 @@
         <v>32</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="42.8" x14ac:dyDescent="0.25">
@@ -851,7 +860,7 @@
         <v>38</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="57.1" x14ac:dyDescent="0.25">
@@ -862,22 +871,22 @@
         <v>39</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>40</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>41</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="42.8" x14ac:dyDescent="0.25">
@@ -888,7 +897,7 @@
         <v>42</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>43</v>
@@ -896,12 +905,14 @@
       <c r="E9" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F9" s="2"/>
+      <c r="F9" s="2" t="s">
+        <v>101</v>
+      </c>
       <c r="G9" s="2" t="s">
         <v>45</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="57.1" x14ac:dyDescent="0.25">
@@ -912,20 +923,22 @@
         <v>46</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>49</v>
+        <v>103</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F10" s="2"/>
+      <c r="F10" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="G10" s="2" t="s">
         <v>48</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="28.55" x14ac:dyDescent="0.25">
@@ -933,23 +946,25 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" t="s">
         <v>51</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2" t="s">
-        <v>53</v>
-      </c>
       <c r="H11" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="42.8" x14ac:dyDescent="0.25">
@@ -957,25 +972,25 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="57.1" x14ac:dyDescent="0.25">
@@ -983,25 +998,25 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="D13" s="3">
         <v>180519</v>
       </c>
       <c r="E13" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>63</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>11</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="42.8" x14ac:dyDescent="0.25">
@@ -1009,25 +1024,25 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>65</v>
       </c>
       <c r="D14" s="3">
         <v>180519</v>
       </c>
       <c r="E14" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="G14" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="G14" s="2" t="s">
-        <v>68</v>
-      </c>
       <c r="H14" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.25">
@@ -1035,25 +1050,25 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>70</v>
       </c>
       <c r="D15" s="3">
         <v>180519</v>
       </c>
       <c r="E15" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F15" s="2" t="s">
-        <v>72</v>
-      </c>
       <c r="G15" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
@@ -1061,25 +1076,25 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="E16" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="F16" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>92</v>
-      </c>
       <c r="H16" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="99.85" x14ac:dyDescent="0.25">
@@ -1087,25 +1102,25 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D17" s="2" t="s">
+      <c r="F17" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="H17" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -1354,13 +1369,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add promise test, what-if and proofs; log row 17
</commit_message>
<xml_diff>
--- a/excel/issues_log.xlsx
+++ b/excel/issues_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DEIVI\Desktop\DA Projects\delivery-performance-analysis\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3E4C9E6-BBBF-4F4C-8B65-EB98902F88B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40D1E6A4-75C3-4262-9FAC-3158038A0674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-27" yWindow="0" windowWidth="20581" windowHeight="19657" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="112">
   <si>
     <t>lines</t>
   </si>
@@ -344,6 +344,24 @@
   </si>
   <si>
     <t>Order Id, Order Item Id</t>
+  </si>
+  <si>
+    <t>Actual days are evenly spread (about 20% each of 2 to 6 days) in Second Class and Standard Class, and always 2 days in First Class</t>
+  </si>
+  <si>
+    <t>Days for shipping (real), Shipping Mode</t>
+  </si>
+  <si>
+    <t>49,888 orders (Second Class 12,256 + Standard Class 37,632) plus 9,602 First Class</t>
+  </si>
+  <si>
+    <t>Report as is; state in the limits that the data looks synthetic and cannot separate carrier from warehouse</t>
+  </si>
+  <si>
+    <t>A natural process would not give equal groups; the finding about the promise still holds because it uses the same data on both sides</t>
+  </si>
+  <si>
+    <t>Promise test</t>
   </si>
 </sst>
 </file>
@@ -1123,15 +1141,31 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
+    <row r="18" spans="1:8" ht="85.6" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>

</xml_diff>